<commit_message>
doc: state of the art
</commit_message>
<xml_diff>
--- a/planning/planning.xlsx
+++ b/planning/planning.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Arnold\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\arnold\master-mse\pa-monkey\documentation\planning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6BCD2D1B-1034-4955-8FBB-673EA959BC79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BE54BAC-DE6A-49B3-9F4F-D5271A7B8DBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{746927A9-20B9-48E5-90D8-AF13595C2FBA}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{746927A9-20B9-48E5-90D8-AF13595C2FBA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,16 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
-  <si>
-    <t>Mapping of equipment/testable interfaces</t>
-  </si>
-  <si>
-    <t>Kickof / Planning</t>
-  </si>
-  <si>
-    <t>Architecture design</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Important dates: 
 start:  17.09.2026
@@ -111,29 +102,26 @@
     <t>Week 18</t>
   </si>
   <si>
-    <t>Doc polishing</t>
-  </si>
-  <si>
-    <t>Slides</t>
-  </si>
-  <si>
-    <t>Monkey Collar integration (bluetooth and power profiling)</t>
-  </si>
-  <si>
-    <t>Gitlab runner setup (if time left)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">State of the art </t>
-  </si>
-  <si>
-    <t>Experimentation:  tools evaluation + zephyr test firmware</t>
+    <t>WP1: Interfaces mapping and requirements analysis</t>
+  </si>
+  <si>
+    <t>WP2: State of the art and testing framework evaluation</t>
+  </si>
+  <si>
+    <t>WP3: Experimentation</t>
+  </si>
+  <si>
+    <t>WP4: Monkey collar testbench implementation</t>
+  </si>
+  <si>
+    <t>WP5: Documentation, delivrables</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -150,6 +138,13 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="7"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -175,7 +170,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="17">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -383,17 +378,31 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -407,9 +416,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -437,6 +447,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -771,7 +784,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6142E62-AA41-4AE0-BB72-D5880E200BD2}">
-  <dimension ref="B2:X19"/>
+  <dimension ref="B2:X15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="5" max="5" width="8.33203125" customWidth="1"/>
@@ -786,7 +799,7 @@
     <row r="2" spans="2:24" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="3" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B3" s="14" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C3" s="15"/>
       <c r="D3" s="15"/>
@@ -818,125 +831,125 @@
     </row>
     <row r="8" spans="2:24" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="9" spans="2:24" x14ac:dyDescent="0.3">
-      <c r="F9" s="4"/>
-      <c r="G9" s="5">
+      <c r="F9" s="3"/>
+      <c r="G9" s="4">
         <v>46282</v>
       </c>
-      <c r="H9" s="5">
+      <c r="H9" s="4">
         <v>46289</v>
       </c>
-      <c r="I9" s="5">
+      <c r="I9" s="4">
         <v>46296</v>
       </c>
-      <c r="J9" s="5">
+      <c r="J9" s="4">
         <v>46303</v>
       </c>
-      <c r="K9" s="5">
+      <c r="K9" s="4">
         <v>46310</v>
       </c>
-      <c r="L9" s="5">
+      <c r="L9" s="4">
         <v>46317</v>
       </c>
-      <c r="M9" s="5">
+      <c r="M9" s="4">
         <v>46324</v>
       </c>
-      <c r="N9" s="5">
+      <c r="N9" s="4">
         <v>46331</v>
       </c>
-      <c r="O9" s="5">
+      <c r="O9" s="4">
         <v>46338</v>
       </c>
-      <c r="P9" s="5">
+      <c r="P9" s="4">
         <v>46345</v>
       </c>
-      <c r="Q9" s="5">
+      <c r="Q9" s="4">
         <v>46352</v>
       </c>
-      <c r="R9" s="5">
+      <c r="R9" s="4">
         <v>46359</v>
       </c>
-      <c r="S9" s="5">
+      <c r="S9" s="4">
         <v>46366</v>
       </c>
-      <c r="T9" s="5">
+      <c r="T9" s="4">
         <v>46373</v>
       </c>
-      <c r="U9" s="5">
+      <c r="U9" s="4">
         <v>46380</v>
       </c>
-      <c r="V9" s="5">
+      <c r="V9" s="4">
         <v>46388</v>
       </c>
-      <c r="W9" s="5">
+      <c r="W9" s="4">
         <v>42743</v>
       </c>
-      <c r="X9" s="6">
+      <c r="X9" s="5">
         <v>46402</v>
       </c>
     </row>
     <row r="10" spans="2:24" x14ac:dyDescent="0.3">
-      <c r="F10" s="7"/>
+      <c r="F10" s="6"/>
       <c r="G10" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="J10" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="K10" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="L10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="J10" s="2" t="s">
+      <c r="M10" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="K10" s="2" t="s">
+      <c r="N10" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="L10" s="2" t="s">
+      <c r="O10" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="M10" s="2" t="s">
+      <c r="P10" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="N10" s="2" t="s">
+      <c r="Q10" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="O10" s="2" t="s">
+      <c r="R10" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="P10" s="2" t="s">
+      <c r="S10" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="Q10" s="2" t="s">
+      <c r="T10" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="R10" s="2" t="s">
+      <c r="U10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="S10" s="2" t="s">
+      <c r="V10" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="T10" s="2" t="s">
+      <c r="W10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="U10" s="2" t="s">
+      <c r="X10" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="V10" s="2" t="s">
+    </row>
+    <row r="11" spans="2:24" x14ac:dyDescent="0.3">
+      <c r="F11" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="W10" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="X10" s="8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="2:24" x14ac:dyDescent="0.3">
-      <c r="F11" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
+      <c r="G11" s="13"/>
+      <c r="H11" s="13"/>
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
@@ -950,19 +963,19 @@
       <c r="S11" s="1"/>
       <c r="T11" s="1"/>
       <c r="U11" s="1"/>
-      <c r="V11" s="12"/>
+      <c r="V11" s="10"/>
       <c r="W11" s="1"/>
-      <c r="X11" s="9"/>
+      <c r="X11" s="8"/>
     </row>
     <row r="12" spans="2:24" x14ac:dyDescent="0.3">
-      <c r="F12" s="7" t="s">
-        <v>0</v>
+      <c r="F12" s="6" t="s">
+        <v>20</v>
       </c>
       <c r="G12" s="1"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="1"/>
-      <c r="J12" s="1"/>
-      <c r="K12" s="1"/>
+      <c r="H12" s="13"/>
+      <c r="I12" s="13"/>
+      <c r="J12" s="13"/>
+      <c r="K12" s="13"/>
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
       <c r="N12" s="1"/>
@@ -973,170 +986,78 @@
       <c r="S12" s="1"/>
       <c r="T12" s="1"/>
       <c r="U12" s="1"/>
-      <c r="V12" s="12"/>
+      <c r="V12" s="10"/>
       <c r="W12" s="1"/>
-      <c r="X12" s="9"/>
+      <c r="X12" s="8"/>
     </row>
     <row r="13" spans="2:24" x14ac:dyDescent="0.3">
-      <c r="F13" s="7" t="s">
-        <v>26</v>
+      <c r="F13" s="6" t="s">
+        <v>21</v>
       </c>
       <c r="G13" s="1"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="1"/>
-      <c r="L13" s="1"/>
-      <c r="M13" s="1"/>
-      <c r="N13" s="1"/>
-      <c r="O13" s="1"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
+      <c r="K13" s="13"/>
+      <c r="L13" s="13"/>
+      <c r="M13" s="13"/>
+      <c r="N13" s="13"/>
+      <c r="O13" s="13"/>
       <c r="P13" s="1"/>
       <c r="Q13" s="1"/>
       <c r="R13" s="1"/>
       <c r="S13" s="1"/>
       <c r="T13" s="1"/>
       <c r="U13" s="1"/>
-      <c r="V13" s="12"/>
+      <c r="V13" s="10"/>
       <c r="W13" s="1"/>
-      <c r="X13" s="9"/>
+      <c r="X13" s="8"/>
     </row>
     <row r="14" spans="2:24" x14ac:dyDescent="0.3">
-      <c r="F14" s="7" t="s">
-        <v>27</v>
+      <c r="F14" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="G14" s="1"/>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
-      <c r="L14" s="3"/>
-      <c r="M14" s="3"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
+      <c r="L14" s="1"/>
+      <c r="M14" s="1"/>
       <c r="N14" s="1"/>
       <c r="O14" s="1"/>
-      <c r="P14" s="1"/>
-      <c r="Q14" s="1"/>
-      <c r="R14" s="1"/>
-      <c r="S14" s="1"/>
-      <c r="T14" s="1"/>
-      <c r="U14" s="1"/>
-      <c r="V14" s="12"/>
+      <c r="P14" s="13"/>
+      <c r="Q14" s="25"/>
+      <c r="R14" s="25"/>
+      <c r="S14" s="25"/>
+      <c r="T14" s="25"/>
+      <c r="U14" s="25"/>
+      <c r="V14" s="10"/>
       <c r="W14" s="1"/>
-      <c r="X14" s="9"/>
-    </row>
-    <row r="15" spans="2:24" x14ac:dyDescent="0.3">
-      <c r="F15" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
-      <c r="J15" s="1"/>
-      <c r="K15" s="1"/>
-      <c r="L15" s="3"/>
-      <c r="M15" s="3"/>
-      <c r="N15" s="3"/>
-      <c r="O15" s="1"/>
-      <c r="P15" s="1"/>
-      <c r="Q15" s="1"/>
-      <c r="R15" s="1"/>
-      <c r="S15" s="1"/>
-      <c r="T15" s="1"/>
-      <c r="U15" s="1"/>
-      <c r="V15" s="12"/>
-      <c r="W15" s="1"/>
-      <c r="X15" s="9"/>
-    </row>
-    <row r="16" spans="2:24" x14ac:dyDescent="0.3">
-      <c r="F16" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="1"/>
-      <c r="J16" s="1"/>
-      <c r="K16" s="1"/>
-      <c r="L16" s="1"/>
-      <c r="M16" s="1"/>
-      <c r="N16" s="3"/>
-      <c r="O16" s="3"/>
-      <c r="P16" s="3"/>
-      <c r="Q16" s="1"/>
-      <c r="R16" s="1"/>
-      <c r="S16" s="1"/>
-      <c r="T16" s="1"/>
-      <c r="U16" s="1"/>
-      <c r="V16" s="12"/>
-      <c r="W16" s="1"/>
-      <c r="X16" s="9"/>
-    </row>
-    <row r="17" spans="6:24" x14ac:dyDescent="0.3">
-      <c r="F17" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-      <c r="J17" s="1"/>
-      <c r="K17" s="1"/>
-      <c r="L17" s="1"/>
-      <c r="M17" s="1"/>
-      <c r="N17" s="1"/>
-      <c r="O17" s="1"/>
-      <c r="P17" s="3"/>
-      <c r="Q17" s="3"/>
-      <c r="R17" s="3"/>
-      <c r="S17" s="1"/>
-      <c r="T17" s="1"/>
-      <c r="U17" s="1"/>
-      <c r="V17" s="12"/>
-      <c r="W17" s="1"/>
-      <c r="X17" s="9"/>
-    </row>
-    <row r="18" spans="6:24" x14ac:dyDescent="0.3">
-      <c r="F18" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G18" s="1"/>
-      <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
-      <c r="K18" s="1"/>
-      <c r="L18" s="1"/>
-      <c r="M18" s="1"/>
-      <c r="N18" s="1"/>
-      <c r="O18" s="1"/>
-      <c r="P18" s="1"/>
-      <c r="Q18" s="1"/>
-      <c r="R18" s="3"/>
-      <c r="S18" s="3"/>
-      <c r="T18" s="3"/>
-      <c r="U18" s="3"/>
-      <c r="V18" s="12"/>
-      <c r="W18" s="3"/>
-      <c r="X18" s="3"/>
-    </row>
-    <row r="19" spans="6:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="F19" s="10" t="s">
+      <c r="X14" s="8"/>
+    </row>
+    <row r="15" spans="2:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="F15" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="G19" s="11"/>
-      <c r="H19" s="11"/>
-      <c r="I19" s="11"/>
-      <c r="J19" s="11"/>
-      <c r="K19" s="11"/>
-      <c r="L19" s="11"/>
-      <c r="M19" s="11"/>
-      <c r="N19" s="11"/>
-      <c r="O19" s="11"/>
-      <c r="P19" s="11"/>
-      <c r="Q19" s="11"/>
-      <c r="R19" s="11"/>
-      <c r="S19" s="11"/>
-      <c r="T19" s="3"/>
-      <c r="U19" s="3"/>
-      <c r="V19" s="13"/>
-      <c r="W19" s="3"/>
-      <c r="X19" s="3"/>
+      <c r="G15" s="23"/>
+      <c r="H15" s="23"/>
+      <c r="I15" s="23"/>
+      <c r="J15" s="23"/>
+      <c r="K15" s="23"/>
+      <c r="L15" s="23"/>
+      <c r="M15" s="23"/>
+      <c r="N15" s="23"/>
+      <c r="O15" s="23"/>
+      <c r="P15" s="23"/>
+      <c r="Q15" s="23"/>
+      <c r="R15" s="23"/>
+      <c r="S15" s="23"/>
+      <c r="T15" s="23"/>
+      <c r="U15" s="23"/>
+      <c r="V15" s="11"/>
+      <c r="W15" s="12"/>
+      <c r="X15" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
doc: advanced on WP1-2
</commit_message>
<xml_diff>
--- a/planning/planning.xlsx
+++ b/planning/planning.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\arnold\master-mse\pa-monkey\documentation\planning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BE54BAC-DE6A-49B3-9F4F-D5271A7B8DBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{339D7383-7902-4C2E-BAAA-DD6B2B372051}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{746927A9-20B9-48E5-90D8-AF13595C2FBA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{746927A9-20B9-48E5-90D8-AF13595C2FBA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="26">
   <si>
     <t>Important dates: 
 start:  17.09.2026
@@ -116,12 +116,18 @@
   <si>
     <t>WP5: Documentation, delivrables</t>
   </si>
+  <si>
+    <t>Expected time</t>
+  </si>
+  <si>
+    <t>Real time</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -149,6 +155,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -403,7 +417,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -420,6 +433,9 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -447,9 +463,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -784,7 +798,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6142E62-AA41-4AE0-BB72-D5880E200BD2}">
-  <dimension ref="B2:X15"/>
+  <dimension ref="B2:X27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="5" max="5" width="8.33203125" customWidth="1"/>
@@ -793,102 +807,116 @@
     <col min="8" max="8" width="12" customWidth="1"/>
     <col min="9" max="9" width="11.5546875" customWidth="1"/>
     <col min="10" max="10" width="12.44140625" customWidth="1"/>
-    <col min="11" max="24" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.5546875" customWidth="1"/>
+    <col min="12" max="12" width="14.109375" customWidth="1"/>
+    <col min="13" max="13" width="14.88671875" customWidth="1"/>
+    <col min="14" max="15" width="14.5546875" customWidth="1"/>
+    <col min="16" max="16" width="14.88671875" customWidth="1"/>
+    <col min="17" max="17" width="15.88671875" customWidth="1"/>
+    <col min="18" max="18" width="13.44140625" customWidth="1"/>
+    <col min="19" max="19" width="14.5546875" customWidth="1"/>
+    <col min="20" max="20" width="14.88671875" customWidth="1"/>
+    <col min="21" max="21" width="14.109375" customWidth="1"/>
+    <col min="22" max="22" width="14.5546875" customWidth="1"/>
+    <col min="23" max="23" width="14.77734375" customWidth="1"/>
+    <col min="24" max="24" width="13.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:24" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="3" spans="2:24" x14ac:dyDescent="0.3">
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="15"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="16"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="18"/>
     </row>
     <row r="4" spans="2:24" x14ac:dyDescent="0.3">
-      <c r="B4" s="17"/>
-      <c r="C4" s="18"/>
-      <c r="D4" s="18"/>
-      <c r="E4" s="19"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="21"/>
     </row>
     <row r="5" spans="2:24" x14ac:dyDescent="0.3">
-      <c r="B5" s="17"/>
-      <c r="C5" s="18"/>
-      <c r="D5" s="18"/>
-      <c r="E5" s="19"/>
+      <c r="B5" s="19"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="21"/>
     </row>
     <row r="6" spans="2:24" x14ac:dyDescent="0.3">
-      <c r="B6" s="17"/>
-      <c r="C6" s="18"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="19"/>
+      <c r="B6" s="19"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
+      <c r="E6" s="21"/>
     </row>
     <row r="7" spans="2:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="20"/>
-      <c r="C7" s="21"/>
-      <c r="D7" s="21"/>
-      <c r="E7" s="22"/>
+      <c r="B7" s="22"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="24"/>
     </row>
     <row r="8" spans="2:24" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="9" spans="2:24" x14ac:dyDescent="0.3">
-      <c r="F9" s="3"/>
-      <c r="G9" s="4">
+      <c r="F9" s="25" t="s">
+        <v>24</v>
+      </c>
+      <c r="G9" s="3">
         <v>46282</v>
       </c>
-      <c r="H9" s="4">
+      <c r="H9" s="3">
         <v>46289</v>
       </c>
-      <c r="I9" s="4">
+      <c r="I9" s="3">
         <v>46296</v>
       </c>
-      <c r="J9" s="4">
+      <c r="J9" s="3">
         <v>46303</v>
       </c>
-      <c r="K9" s="4">
+      <c r="K9" s="3">
         <v>46310</v>
       </c>
-      <c r="L9" s="4">
+      <c r="L9" s="3">
         <v>46317</v>
       </c>
-      <c r="M9" s="4">
+      <c r="M9" s="3">
         <v>46324</v>
       </c>
-      <c r="N9" s="4">
+      <c r="N9" s="3">
         <v>46331</v>
       </c>
-      <c r="O9" s="4">
+      <c r="O9" s="3">
         <v>46338</v>
       </c>
-      <c r="P9" s="4">
+      <c r="P9" s="3">
         <v>46345</v>
       </c>
-      <c r="Q9" s="4">
+      <c r="Q9" s="3">
         <v>46352</v>
       </c>
-      <c r="R9" s="4">
+      <c r="R9" s="3">
         <v>46359</v>
       </c>
-      <c r="S9" s="4">
+      <c r="S9" s="3">
         <v>46366</v>
       </c>
-      <c r="T9" s="4">
+      <c r="T9" s="3">
         <v>46373</v>
       </c>
-      <c r="U9" s="4">
+      <c r="U9" s="3">
         <v>46380</v>
       </c>
-      <c r="V9" s="4">
+      <c r="V9" s="3">
         <v>46388</v>
       </c>
-      <c r="W9" s="4">
+      <c r="W9" s="3">
         <v>42743</v>
       </c>
-      <c r="X9" s="5">
+      <c r="X9" s="4">
         <v>46402</v>
       </c>
     </row>
     <row r="10" spans="2:24" x14ac:dyDescent="0.3">
-      <c r="F10" s="6"/>
+      <c r="F10" s="5"/>
       <c r="G10" s="2" t="s">
         <v>1</v>
       </c>
@@ -940,16 +968,16 @@
       <c r="W10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="X10" s="7" t="s">
+      <c r="X10" s="6" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="11" spans="2:24" x14ac:dyDescent="0.3">
-      <c r="F11" s="6" t="s">
+      <c r="F11" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="G11" s="13"/>
-      <c r="H11" s="13"/>
+      <c r="G11" s="12"/>
+      <c r="H11" s="12"/>
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
@@ -963,19 +991,19 @@
       <c r="S11" s="1"/>
       <c r="T11" s="1"/>
       <c r="U11" s="1"/>
-      <c r="V11" s="10"/>
+      <c r="V11" s="9"/>
       <c r="W11" s="1"/>
-      <c r="X11" s="8"/>
+      <c r="X11" s="7"/>
     </row>
     <row r="12" spans="2:24" x14ac:dyDescent="0.3">
-      <c r="F12" s="6" t="s">
+      <c r="F12" s="5" t="s">
         <v>20</v>
       </c>
       <c r="G12" s="1"/>
-      <c r="H12" s="13"/>
-      <c r="I12" s="13"/>
-      <c r="J12" s="13"/>
-      <c r="K12" s="13"/>
+      <c r="H12" s="12"/>
+      <c r="I12" s="12"/>
+      <c r="J12" s="12"/>
+      <c r="K12" s="12"/>
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
       <c r="N12" s="1"/>
@@ -986,35 +1014,35 @@
       <c r="S12" s="1"/>
       <c r="T12" s="1"/>
       <c r="U12" s="1"/>
-      <c r="V12" s="10"/>
+      <c r="V12" s="9"/>
       <c r="W12" s="1"/>
-      <c r="X12" s="8"/>
+      <c r="X12" s="7"/>
     </row>
     <row r="13" spans="2:24" x14ac:dyDescent="0.3">
-      <c r="F13" s="6" t="s">
+      <c r="F13" s="5" t="s">
         <v>21</v>
       </c>
       <c r="G13" s="1"/>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
-      <c r="K13" s="13"/>
-      <c r="L13" s="13"/>
-      <c r="M13" s="13"/>
-      <c r="N13" s="13"/>
-      <c r="O13" s="13"/>
+      <c r="K13" s="12"/>
+      <c r="L13" s="12"/>
+      <c r="M13" s="12"/>
+      <c r="N13" s="12"/>
+      <c r="O13" s="12"/>
       <c r="P13" s="1"/>
       <c r="Q13" s="1"/>
       <c r="R13" s="1"/>
       <c r="S13" s="1"/>
       <c r="T13" s="1"/>
       <c r="U13" s="1"/>
-      <c r="V13" s="10"/>
+      <c r="V13" s="9"/>
       <c r="W13" s="1"/>
-      <c r="X13" s="8"/>
+      <c r="X13" s="7"/>
     </row>
     <row r="14" spans="2:24" x14ac:dyDescent="0.3">
-      <c r="F14" s="6" t="s">
+      <c r="F14" s="5" t="s">
         <v>22</v>
       </c>
       <c r="G14" s="1"/>
@@ -1026,38 +1054,270 @@
       <c r="M14" s="1"/>
       <c r="N14" s="1"/>
       <c r="O14" s="1"/>
-      <c r="P14" s="13"/>
-      <c r="Q14" s="25"/>
-      <c r="R14" s="25"/>
-      <c r="S14" s="25"/>
-      <c r="T14" s="25"/>
-      <c r="U14" s="25"/>
-      <c r="V14" s="10"/>
+      <c r="P14" s="12"/>
+      <c r="Q14" s="15"/>
+      <c r="R14" s="15"/>
+      <c r="S14" s="15"/>
+      <c r="T14" s="15"/>
+      <c r="U14" s="15"/>
+      <c r="V14" s="9"/>
       <c r="W14" s="1"/>
-      <c r="X14" s="8"/>
+      <c r="X14" s="7"/>
     </row>
     <row r="15" spans="2:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="F15" s="9" t="s">
+      <c r="F15" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="G15" s="23"/>
-      <c r="H15" s="23"/>
-      <c r="I15" s="23"/>
-      <c r="J15" s="23"/>
-      <c r="K15" s="23"/>
-      <c r="L15" s="23"/>
-      <c r="M15" s="23"/>
-      <c r="N15" s="23"/>
-      <c r="O15" s="23"/>
-      <c r="P15" s="23"/>
-      <c r="Q15" s="23"/>
-      <c r="R15" s="23"/>
-      <c r="S15" s="23"/>
-      <c r="T15" s="23"/>
-      <c r="U15" s="23"/>
-      <c r="V15" s="11"/>
-      <c r="W15" s="12"/>
-      <c r="X15" s="24"/>
+      <c r="G15" s="13"/>
+      <c r="H15" s="13"/>
+      <c r="I15" s="13"/>
+      <c r="J15" s="13"/>
+      <c r="K15" s="13"/>
+      <c r="L15" s="13"/>
+      <c r="M15" s="13"/>
+      <c r="N15" s="13"/>
+      <c r="O15" s="13"/>
+      <c r="P15" s="13"/>
+      <c r="Q15" s="13"/>
+      <c r="R15" s="13"/>
+      <c r="S15" s="13"/>
+      <c r="T15" s="13"/>
+      <c r="U15" s="13"/>
+      <c r="V15" s="10"/>
+      <c r="W15" s="11"/>
+      <c r="X15" s="14"/>
+    </row>
+    <row r="20" spans="6:24" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="21" spans="6:24" x14ac:dyDescent="0.3">
+      <c r="F21" s="25" t="s">
+        <v>25</v>
+      </c>
+      <c r="G21" s="3">
+        <v>46282</v>
+      </c>
+      <c r="H21" s="3">
+        <v>46289</v>
+      </c>
+      <c r="I21" s="3">
+        <v>46296</v>
+      </c>
+      <c r="J21" s="3">
+        <v>46303</v>
+      </c>
+      <c r="K21" s="3">
+        <v>46310</v>
+      </c>
+      <c r="L21" s="3">
+        <v>46317</v>
+      </c>
+      <c r="M21" s="3">
+        <v>46324</v>
+      </c>
+      <c r="N21" s="3">
+        <v>46331</v>
+      </c>
+      <c r="O21" s="3">
+        <v>46338</v>
+      </c>
+      <c r="P21" s="3">
+        <v>46345</v>
+      </c>
+      <c r="Q21" s="3">
+        <v>46352</v>
+      </c>
+      <c r="R21" s="3">
+        <v>46359</v>
+      </c>
+      <c r="S21" s="3">
+        <v>46366</v>
+      </c>
+      <c r="T21" s="3">
+        <v>46373</v>
+      </c>
+      <c r="U21" s="3">
+        <v>46380</v>
+      </c>
+      <c r="V21" s="3">
+        <v>46388</v>
+      </c>
+      <c r="W21" s="3">
+        <v>42743</v>
+      </c>
+      <c r="X21" s="4">
+        <v>46402</v>
+      </c>
+    </row>
+    <row r="22" spans="6:24" x14ac:dyDescent="0.3">
+      <c r="F22" s="5"/>
+      <c r="G22" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="K22" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="L22" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="M22" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="N22" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="O22" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="P22" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q22" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="R22" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S22" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="T22" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="U22" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="V22" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="W22" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="X22" s="6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="23" spans="6:24" x14ac:dyDescent="0.3">
+      <c r="F23" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="G23" s="12"/>
+      <c r="H23" s="12"/>
+      <c r="I23" s="12"/>
+      <c r="J23" s="1"/>
+      <c r="K23" s="1"/>
+      <c r="L23" s="1"/>
+      <c r="M23" s="1"/>
+      <c r="N23" s="1"/>
+      <c r="O23" s="1"/>
+      <c r="P23" s="1"/>
+      <c r="Q23" s="1"/>
+      <c r="R23" s="1"/>
+      <c r="S23" s="1"/>
+      <c r="T23" s="1"/>
+      <c r="U23" s="1"/>
+      <c r="V23" s="9"/>
+      <c r="W23" s="1"/>
+      <c r="X23" s="7"/>
+    </row>
+    <row r="24" spans="6:24" x14ac:dyDescent="0.3">
+      <c r="F24" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="G24" s="1"/>
+      <c r="H24" s="1"/>
+      <c r="I24" s="12"/>
+      <c r="J24" s="1"/>
+      <c r="K24" s="1"/>
+      <c r="L24" s="1"/>
+      <c r="M24" s="1"/>
+      <c r="N24" s="1"/>
+      <c r="O24" s="1"/>
+      <c r="P24" s="1"/>
+      <c r="Q24" s="1"/>
+      <c r="R24" s="1"/>
+      <c r="S24" s="1"/>
+      <c r="T24" s="1"/>
+      <c r="U24" s="1"/>
+      <c r="V24" s="9"/>
+      <c r="W24" s="1"/>
+      <c r="X24" s="7"/>
+    </row>
+    <row r="25" spans="6:24" x14ac:dyDescent="0.3">
+      <c r="F25" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="G25" s="1"/>
+      <c r="H25" s="1"/>
+      <c r="I25" s="1"/>
+      <c r="J25" s="1"/>
+      <c r="K25" s="1"/>
+      <c r="L25" s="1"/>
+      <c r="M25" s="1"/>
+      <c r="N25" s="1"/>
+      <c r="O25" s="1"/>
+      <c r="P25" s="1"/>
+      <c r="Q25" s="1"/>
+      <c r="R25" s="1"/>
+      <c r="S25" s="1"/>
+      <c r="T25" s="1"/>
+      <c r="U25" s="1"/>
+      <c r="V25" s="9"/>
+      <c r="W25" s="1"/>
+      <c r="X25" s="7"/>
+    </row>
+    <row r="26" spans="6:24" x14ac:dyDescent="0.3">
+      <c r="F26" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G26" s="1"/>
+      <c r="H26" s="1"/>
+      <c r="I26" s="1"/>
+      <c r="J26" s="1"/>
+      <c r="K26" s="1"/>
+      <c r="L26" s="1"/>
+      <c r="M26" s="1"/>
+      <c r="N26" s="1"/>
+      <c r="O26" s="1"/>
+      <c r="P26" s="1"/>
+      <c r="Q26" s="1"/>
+      <c r="R26" s="1"/>
+      <c r="S26" s="1"/>
+      <c r="T26" s="1"/>
+      <c r="U26" s="1"/>
+      <c r="V26" s="9"/>
+      <c r="W26" s="1"/>
+      <c r="X26" s="7"/>
+    </row>
+    <row r="27" spans="6:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="F27" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="G27" s="13"/>
+      <c r="H27" s="13"/>
+      <c r="I27" s="13"/>
+      <c r="J27" s="13"/>
+      <c r="K27" s="13"/>
+      <c r="L27" s="13"/>
+      <c r="M27" s="13"/>
+      <c r="N27" s="13"/>
+      <c r="O27" s="13"/>
+      <c r="P27" s="13"/>
+      <c r="Q27" s="13"/>
+      <c r="R27" s="13"/>
+      <c r="S27" s="13"/>
+      <c r="T27" s="13"/>
+      <c r="U27" s="13"/>
+      <c r="V27" s="10"/>
+      <c r="W27" s="11"/>
+      <c r="X27" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>